<commit_message>
Wire charts natively into both workbooks
Phase 1 gains a Charts tab with four native Excel charts driven by the
data tabs: cumulative revenue vs plan vs prior year, gross margin
columns vs the 61.6% budget line, utilization columns with per-person
target markers, and sales by customer. Phase 2 gains a Coverage Chart
tab: stacked backlog + weighted-pipeline areas under the Base forecast
line, with a 1/0 toggle cell that includes or excludes the pipeline and
live coverage/gap readout cells. All chart data blocks are formulas
referencing the source tabs, so edits to jobs, bids, probabilities, or
the scenario selector redraw the charts.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145i7FWr3AQEo26DBw1x2c4
</commit_message>
<xml_diff>
--- a/model/CVR_Model_Phase1_Baseline.xlsx
+++ b/model/CVR_Model_Phase1_Baseline.xlsx
@@ -18,6 +18,7 @@
     <sheet name="HWC EPC Baseline" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Realization" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Checks &amp; Open Items" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Charts" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -226,6 +227,638 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumulative revenue — Actual vs Plan vs Prior Year ($K)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!A42</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Charts'!$B$41:$G$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$42:$G$42</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!A43</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Charts'!$B$41:$G$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$43:$G$43</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!A44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Charts'!$B$41:$G$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$44:$G$44</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>$K cumulative</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gross margin by month vs 61.6% budget assumption</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!A47</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$B$41:$G$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$47:$G$47</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!A48</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Charts'!$B$41:$G$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$48:$G$48</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.8"/>
+          <min val="-0.6"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.8"/>
+          <min val="-0.6"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Billable utilization vs target, by person (YTD)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Roster &amp; Hours'!F4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Roster &amp; Hours'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Roster &amp; Hours'!$F$5:$F$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Roster &amp; Hours'!J4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="dash"/>
+            <size val="12"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Roster &amp; Hours'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Roster &amp; Hours'!$J$5:$J$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="210"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.05"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="210"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.05"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sales by customer — YTD June 2026 ($)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cash Flow &amp; Customers'!$A$17:$A$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cash Flow &amp; Customers'!$B$17:$B$23</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -517,7 +1150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -642,62 +1275,76 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Charts               — native charts wired to the data tabs (revenue vs plan/PY, gross margin,</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         utilization vs target, sales by customer). Edit data; charts redraw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>COLOR KEY</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Blue  = input / assumption you can change</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Black = calculated or sourced from a document</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Blue  = input / assumption you can change</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Black = calculated or sourced from a document</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Orange italics = assumption that needs confirmation</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  data/CVR_Rate_Sheet_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  data/CVR_EPC_KPI_2026-07-11.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  data/CVR_Rate_Sheet_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  data/CVR_EPC_KPI_2026-07-11.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t xml:space="preserve">  data/CVR_Financial_Statements_2026-06-30.pdf</t>
         </is>
@@ -1514,6 +2161,232 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Charts — wired to the data tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Native Excel charts driven by cell values: edit the data tabs and these redraw. Data blocks feeding them start at row 40.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>CHART DATA — cumulative revenue ($K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jan 26</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Feb 26</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Mar 26</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Apr 26</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>May 26</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Actual (cumulative)</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>'Baseline P&amp;L'!B5</f>
+        <v/>
+      </c>
+      <c r="C42">
+        <f>B42+'Baseline P&amp;L'!C5</f>
+        <v/>
+      </c>
+      <c r="D42">
+        <f>C42+'Baseline P&amp;L'!D5</f>
+        <v/>
+      </c>
+      <c r="E42">
+        <f>D42+'Baseline P&amp;L'!E5</f>
+        <v/>
+      </c>
+      <c r="F42">
+        <f>E42+'Baseline P&amp;L'!F5</f>
+        <v/>
+      </c>
+      <c r="G42">
+        <f>F42+'Baseline P&amp;L'!G5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Plan (cumulative)</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>'Baseline P&amp;L'!B14</f>
+        <v/>
+      </c>
+      <c r="C43">
+        <f>B43+'Baseline P&amp;L'!C14</f>
+        <v/>
+      </c>
+      <c r="D43">
+        <f>C43+'Baseline P&amp;L'!D14</f>
+        <v/>
+      </c>
+      <c r="E43">
+        <f>D43+'Baseline P&amp;L'!E14</f>
+        <v/>
+      </c>
+      <c r="F43">
+        <f>E43+'Baseline P&amp;L'!F14</f>
+        <v/>
+      </c>
+      <c r="G43">
+        <f>F43+'Baseline P&amp;L'!G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Prior year (pace)</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="C44" t="n">
+        <v>133</v>
+      </c>
+      <c r="D44" t="n">
+        <v>199.6</v>
+      </c>
+      <c r="E44" t="n">
+        <v>266.1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>332.6</v>
+      </c>
+      <c r="G44" t="n">
+        <v>399.1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>CHART DATA — gross margin %</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B47" s="24">
+        <f>'Baseline P&amp;L'!B8</f>
+        <v/>
+      </c>
+      <c r="C47" s="24">
+        <f>'Baseline P&amp;L'!C8</f>
+        <v/>
+      </c>
+      <c r="D47" s="24">
+        <f>'Baseline P&amp;L'!D8</f>
+        <v/>
+      </c>
+      <c r="E47" s="24">
+        <f>'Baseline P&amp;L'!E8</f>
+        <v/>
+      </c>
+      <c r="F47" s="24">
+        <f>'Baseline P&amp;L'!F8</f>
+        <v/>
+      </c>
+      <c r="G47" s="24">
+        <f>'Baseline P&amp;L'!G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Budget assumption</t>
+        </is>
+      </c>
+      <c r="B48" s="24" t="n">
+        <v>0.6157</v>
+      </c>
+      <c r="C48" s="24" t="n">
+        <v>0.6157</v>
+      </c>
+      <c r="D48" s="24" t="n">
+        <v>0.6157</v>
+      </c>
+      <c r="E48" s="24" t="n">
+        <v>0.6157</v>
+      </c>
+      <c r="F48" s="24" t="n">
+        <v>0.6157</v>
+      </c>
+      <c r="G48" s="24" t="n">
+        <v>0.6157</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add Labor Cost tab from COINS timesheet cost report (per-person rates)
Incorporate data/CVR_Timesheet_Costs_Jul2026_JC016755.pdf: per-person
standard cost rates (Roy Pierce $149.57 down to Collin Allen $51.11),
consistent to the penny across every timesheet line. New Labor Cost tab
computes loaded cost (raw x 1+burden) and margin/multiplier by role
against the bill card, with a blended weighted-by-hours line. Documents
the assessment that these are base/pay rates (burden-exclusive) with two
tells: GL books burden as separate OpEx (not COGS), and PTO/holiday
hours are booked at the same per-person rate. Rates cluster by grade,
validating the data.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145i7FWr3AQEo26DBw1x2c4
</commit_message>
<xml_diff>
--- a/model/CVR_Model_Phase1_Baseline.xlsx
+++ b/model/CVR_Model_Phase1_Baseline.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Rates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Roster &amp; Hours" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Baseline P&amp;L" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="GL Income Stmt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Balance Sheet" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cash Flow &amp; Customers" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="HWC EPC Baseline" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Realization" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Checks &amp; Open Items" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Charts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster &amp; Hours" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labor Cost" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline P&amp;L" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GL Income Stmt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow &amp; Customers" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HWC EPC Baseline" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realization" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Open Items" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,8 +35,8 @@
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="170" formatCode="#,##0.0;(#,##0.0)"/>
-    <numFmt numFmtId="171" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="171" formatCode="#,##0.0;(#,##0.0)"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -115,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,7 +141,9 @@
     <xf numFmtId="168" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,9 +151,8 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -230,13 +232,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -259,7 +261,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="2A78D6"/>
               </a:solidFill>
@@ -269,7 +271,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -295,7 +297,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
               <a:solidFill>
                 <a:srgbClr val="898781"/>
               </a:solidFill>
@@ -305,7 +307,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -331,7 +333,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
               <a:solidFill>
                 <a:srgbClr val="898781"/>
               </a:solidFill>
@@ -341,7 +343,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -382,8 +384,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -409,13 +411,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -439,10 +441,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -472,7 +474,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
               <a:solidFill>
                 <a:srgbClr val="898781"/>
               </a:solidFill>
@@ -482,7 +484,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -551,13 +553,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -581,10 +583,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -614,7 +616,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -623,7 +625,7 @@
             <symbol val="dash"/>
             <size val="12"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -692,13 +694,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -717,10 +719,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -769,7 +771,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -784,9 +786,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -806,9 +808,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -828,9 +830,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -850,9 +852,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1150,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1228,125 +1230,139 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Baseline P&amp;L         — CVR monthly actuals vs budget, Jan–Jun 2026 (Jan–May per KPI report, June per GL).</t>
+          <t xml:space="preserve">  Labor Cost           — per-person standard cost rates (COINS timesheet report), loaded cost, and margin by role.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GL Income Stmt       — full line-item income statement, June and YTD, actual vs budget vs prior year.</t>
+          <t xml:space="preserve">  Baseline P&amp;L         — CVR monthly actuals vs budget, Jan–Jun 2026 (Jan–May per KPI report, June per GL).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Balance Sheet        — 6/30/2026 vs one year ago vs annual budget.</t>
+          <t xml:space="preserve">  GL Income Stmt       — full line-item income statement, June and YTD, actual vs budget vs prior year.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash Flow &amp; Customers— six-month cash flow summary and sales by customer (incl. intercompany).</t>
+          <t xml:space="preserve">  Balance Sheet        — 6/30/2026 vs one year ago vs annual budget.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HWC EPC Baseline     — EPC line financials for context.</t>
+          <t xml:space="preserve">  Cash Flow &amp; Customers— six-month cash flow summary and sales by customer (incl. intercompany).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Realization          — the $/hr and labor-multiplier gap analysis plus the utilization × realization grid.</t>
+          <t xml:space="preserve">  HWC EPC Baseline     — EPC line financials for context.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Checks &amp; Open Items  — tie-outs across all three sources and remaining open questions.</t>
+          <t xml:space="preserve">  Realization          — the $/hr and labor-multiplier gap analysis plus the utilization × realization grid.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Charts               — native charts wired to the data tabs (revenue vs plan/PY, gross margin,</t>
+          <t xml:space="preserve">  Checks &amp; Open Items  — tie-outs across all three sources and remaining open questions.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Charts               — native charts wired to the data tabs (revenue vs plan/PY, gross margin,</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t xml:space="preserve">                         utilization vs target, sales by customer). Edit data; charts redraw.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>COLOR KEY</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Blue  = input / assumption you can change</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Black = calculated or sourced from a document</t>
+          <t xml:space="preserve">  Blue  = input / assumption you can change</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Black = calculated or sourced from a document</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Orange italics = assumption that needs confirmation</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  data/CVR_Rate_Sheet_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  data/CVR_EPC_KPI_2026-07-11.pdf</t>
+          <t xml:space="preserve">  data/CVR_Rate_Sheet_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t xml:space="preserve">  data/CVR_EPC_KPI_2026-07-11.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t xml:space="preserve">  data/CVR_Financial_Statements_2026-06-30.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  data/CVR_Timesheet_Costs_Jul2026_JC016755.pdf</t>
         </is>
       </c>
     </row>
@@ -1356,6 +1372,164 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HWC EPC — Baseline, January–May 2026 (all figures $K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Context for the engineering P&amp;L: design quality and constructability directly affect these outcomes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>HWC EPC ($K)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>732.2</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>207.7</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>-321</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>-125.1</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>678.6</v>
+      </c>
+      <c r="G5" s="24">
+        <f>SUM(B5:F5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Net Profit / (Loss)</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>-318.3</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>-346.9</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>-672.8</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>-656.5</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>-114.8</v>
+      </c>
+      <c r="G6" s="24">
+        <f>SUM(B6:F6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Net margin % (YTD)</t>
+        </is>
+      </c>
+      <c r="G7" s="26">
+        <f>G6/G5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Negative revenue in March and April are billing adjustments/write-downs per the KPI report charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Active EPC scorecard jobs (7/11/2026): 4 substation projects, PO $4.3M–$6.6M, plan margins 12.7%–16.4%,</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>cost variance +3.6% to −19.8%. Engineering share of paired EPC pursuits runs ~4–5% of EPC job value.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1424,7 +1598,7 @@
           <t>Adjustment factor to June 30</t>
         </is>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="31">
         <f>Assumptions!B8</f>
         <v/>
       </c>
@@ -1472,7 +1646,7 @@
           <t>Value at card rates, Jan–Jun ($K)</t>
         </is>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="23">
         <f>B7*B8/1000</f>
         <v/>
       </c>
@@ -1488,7 +1662,7 @@
           <t>Actual revenue, Jan–Jun ($K)</t>
         </is>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="23">
         <f>'GL Income Stmt'!E5/1000</f>
         <v/>
       </c>
@@ -1536,7 +1710,7 @@
           <t>Unexplained gap ($K)</t>
         </is>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="23">
         <f>B9-B10</f>
         <v/>
       </c>
@@ -1552,7 +1726,7 @@
           <t>Direct labor cost ($K, GL)</t>
         </is>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="23">
         <f>'GL Income Stmt'!E7/1000</f>
         <v/>
       </c>
@@ -1584,7 +1758,7 @@
           <t>Labor multiplier — actual (rev ÷ direct labor)</t>
         </is>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="21">
         <f>B10/B14</f>
         <v/>
       </c>
@@ -1600,7 +1774,7 @@
           <t>Labor multiplier — budget</t>
         </is>
       </c>
-      <c r="B17" s="30">
+      <c r="B17" s="21">
         <f>'GL Income Stmt'!F5/'GL Income Stmt'!F7</f>
         <v/>
       </c>
@@ -1623,7 +1797,7 @@
           <t>Unbilled WIP / billing lag ($K)</t>
         </is>
       </c>
-      <c r="B20" s="31" t="n">
+      <c r="B20" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1633,7 +1807,7 @@
           <t>Write-offs &amp; discounts ($K)</t>
         </is>
       </c>
-      <c r="B21" s="31" t="n">
+      <c r="B21" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1643,7 +1817,7 @@
           <t>Intercompany work at reduced rates ($K)</t>
         </is>
       </c>
-      <c r="B22" s="31" t="n">
+      <c r="B22" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1653,7 +1827,7 @@
           <t>Other / unreconciled ($K)</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n">
+      <c r="B23" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1663,7 +1837,7 @@
           <t>Decomposition vs gap</t>
         </is>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="33">
         <f>SUM(B20:B23)-B13</f>
         <v/>
       </c>
@@ -1686,99 +1860,99 @@
           <t>Utilization ↓ / Realization →</t>
         </is>
       </c>
-      <c r="B28" s="33" t="n">
+      <c r="B28" s="34" t="n">
         <v>0.6</v>
       </c>
-      <c r="C28" s="33" t="n">
+      <c r="C28" s="34" t="n">
         <v>0.75</v>
       </c>
-      <c r="D28" s="33" t="n">
+      <c r="D28" s="34" t="n">
         <v>0.9</v>
       </c>
-      <c r="E28" s="33" t="n">
+      <c r="E28" s="34" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="n">
+      <c r="A29" s="34" t="n">
         <v>0.59</v>
       </c>
-      <c r="B29" s="34">
+      <c r="B29" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A29*B$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="C29" s="34">
+      <c r="C29" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A29*C$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="D29" s="34">
+      <c r="D29" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A29*D$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="E29" s="34">
+      <c r="E29" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A29*E$28*$B$8/1000</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="33" t="n">
+      <c r="A30" s="34" t="n">
         <v>0.65</v>
       </c>
-      <c r="B30" s="34">
+      <c r="B30" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A30*B$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="C30" s="34">
+      <c r="C30" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A30*C$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="D30" s="34">
+      <c r="D30" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A30*D$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="E30" s="34">
+      <c r="E30" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A30*E$28*$B$8/1000</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="33" t="n">
+      <c r="A31" s="34" t="n">
         <v>0.7</v>
       </c>
-      <c r="B31" s="34">
+      <c r="B31" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A31*B$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="C31" s="34">
+      <c r="C31" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A31*C$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="D31" s="34">
+      <c r="D31" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A31*D$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A31*E$28*$B$8/1000</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="33" t="n">
+      <c r="A32" s="34" t="n">
         <v>0.75</v>
       </c>
-      <c r="B32" s="34">
+      <c r="B32" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A32*B$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="C32" s="34">
+      <c r="C32" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A32*C$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="D32" s="34">
+      <c r="D32" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A32*D$28*$B$8/1000</f>
         <v/>
       </c>
-      <c r="E32" s="34">
+      <c r="E32" s="35">
         <f>Assumptions!B7*Assumptions!B5*$A32*E$28*$B$8/1000</f>
         <v/>
       </c>
@@ -1823,7 +1997,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1873,11 +2047,11 @@
           <t>CVR revenue YTD Jun ($K) vs GL</t>
         </is>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="23">
         <f>'Baseline P&amp;L'!H5</f>
         <v/>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="23" t="n">
         <v>551</v>
       </c>
       <c r="D5" s="5">
@@ -1891,11 +2065,11 @@
           <t>CVR gross profit YTD Jun ($K) vs GL</t>
         </is>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="23">
         <f>'Baseline P&amp;L'!H7</f>
         <v/>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="23" t="n">
         <v>122.5</v>
       </c>
       <c r="D6" s="5">
@@ -1909,11 +2083,11 @@
           <t>CVR net income YTD Jun ($K) vs GL</t>
         </is>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="23">
         <f>'Baseline P&amp;L'!H10</f>
         <v/>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="23" t="n">
         <v>-320.5</v>
       </c>
       <c r="D7" s="5">
@@ -1927,11 +2101,11 @@
           <t>KPI Jan–May revenue ($K) vs GL (YTD−Jun)</t>
         </is>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="23">
         <f>SUM('Baseline P&amp;L'!B5:F5)</f>
         <v/>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="23" t="n">
         <v>426.7</v>
       </c>
       <c r="D8" s="5">
@@ -1945,11 +2119,11 @@
           <t>KPI Jan–May net income ($K) vs GL (YTD−Jun)</t>
         </is>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="23">
         <f>SUM('Baseline P&amp;L'!B10:F10)</f>
         <v/>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="23" t="n">
         <v>-304.7</v>
       </c>
       <c r="D9" s="5">
@@ -1999,11 +2173,11 @@
           <t>EPC revenue YTD May ($K)</t>
         </is>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="23">
         <f>'HWC EPC Baseline'!G5</f>
         <v/>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="23" t="n">
         <v>1172.4</v>
       </c>
       <c r="D12" s="5">
@@ -2017,11 +2191,11 @@
           <t>EPC net profit YTD May ($K)</t>
         </is>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="23">
         <f>'HWC EPC Baseline'!G6</f>
         <v/>
       </c>
-      <c r="C13" s="21" t="n">
+      <c r="C13" s="23" t="n">
         <v>-2109.3</v>
       </c>
       <c r="D13" s="5">
@@ -2035,11 +2209,11 @@
           <t>Billable hours YTD</t>
         </is>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="23">
         <f>'Roster &amp; Hours'!I18</f>
         <v/>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="23" t="n">
         <v>4747</v>
       </c>
       <c r="D14" s="5">
@@ -2164,7 +2338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2334,27 +2508,27 @@
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="B47" s="24">
+      <c r="B47" s="26">
         <f>'Baseline P&amp;L'!B8</f>
         <v/>
       </c>
-      <c r="C47" s="24">
+      <c r="C47" s="26">
         <f>'Baseline P&amp;L'!C8</f>
         <v/>
       </c>
-      <c r="D47" s="24">
+      <c r="D47" s="26">
         <f>'Baseline P&amp;L'!D8</f>
         <v/>
       </c>
-      <c r="E47" s="24">
+      <c r="E47" s="26">
         <f>'Baseline P&amp;L'!E8</f>
         <v/>
       </c>
-      <c r="F47" s="24">
+      <c r="F47" s="26">
         <f>'Baseline P&amp;L'!F8</f>
         <v/>
       </c>
-      <c r="G47" s="24">
+      <c r="G47" s="26">
         <f>'Baseline P&amp;L'!G8</f>
         <v/>
       </c>
@@ -2365,22 +2539,22 @@
           <t>Budget assumption</t>
         </is>
       </c>
-      <c r="B48" s="24" t="n">
+      <c r="B48" s="26" t="n">
         <v>0.6157</v>
       </c>
-      <c r="C48" s="24" t="n">
+      <c r="C48" s="26" t="n">
         <v>0.6157</v>
       </c>
-      <c r="D48" s="24" t="n">
+      <c r="D48" s="26" t="n">
         <v>0.6157</v>
       </c>
-      <c r="E48" s="24" t="n">
+      <c r="E48" s="26" t="n">
         <v>0.6157</v>
       </c>
-      <c r="F48" s="24" t="n">
+      <c r="F48" s="26" t="n">
         <v>0.6157</v>
       </c>
-      <c r="G48" s="24" t="n">
+      <c r="G48" s="26" t="n">
         <v>0.6157</v>
       </c>
     </row>
@@ -3481,6 +3655,533 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Labor Cost — standard rates and margin by person</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cost rates from COINS Timesheet Costs Report (JC016755), Jul 2026. Loaded cost = raw × (1 + burden). Burden on Assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Billing classification</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Bill rate / hr</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Raw cost / hr</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Loaded cost / hr</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Margin / hr (bill − loaded)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Cost multiplier (bill ÷ loaded)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Billable value @ card</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Roy Pierce</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Principal Engineer</t>
+        </is>
+      </c>
+      <c r="C5" s="12">
+        <f>Rates!B16</f>
+        <v/>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>149.57</v>
+      </c>
+      <c r="E5" s="12">
+        <f>D5*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F5" s="12">
+        <f>C5-E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="21">
+        <f>C5/E5</f>
+        <v/>
+      </c>
+      <c r="H5" s="14">
+        <f>'Roster &amp; Hours'!L12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Hayley Worthen</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Senior Engineer</t>
+        </is>
+      </c>
+      <c r="C6" s="12">
+        <f>Rates!B15</f>
+        <v/>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>138.05</v>
+      </c>
+      <c r="E6" s="12">
+        <f>D6*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>C6-E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="21">
+        <f>C6/E6</f>
+        <v/>
+      </c>
+      <c r="H6" s="14">
+        <f>'Roster &amp; Hours'!L8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Bhkti Patel</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Engineer III</t>
+        </is>
+      </c>
+      <c r="C7" s="12">
+        <f>Rates!B13</f>
+        <v/>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="E7" s="12">
+        <f>D7*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F7" s="12">
+        <f>C7-E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>C7/E7</f>
+        <v/>
+      </c>
+      <c r="H7" s="14">
+        <f>'Roster &amp; Hours'!L6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Francis Wagner</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Engineer III</t>
+        </is>
+      </c>
+      <c r="C8" s="12">
+        <f>Rates!B13</f>
+        <v/>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="E8" s="12">
+        <f>D8*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>C8-E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="21">
+        <f>C8/E8</f>
+        <v/>
+      </c>
+      <c r="H8" s="14">
+        <f>'Roster &amp; Hours'!L9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Kevin Metts</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Designer II</t>
+        </is>
+      </c>
+      <c r="C9" s="12">
+        <f>Rates!B9</f>
+        <v/>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>92.39</v>
+      </c>
+      <c r="E9" s="12">
+        <f>D9*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="12">
+        <f>C9-E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>C9/E9</f>
+        <v/>
+      </c>
+      <c r="H9" s="14">
+        <f>'Roster &amp; Hours'!L11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Craig Peterson</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Engineer I</t>
+        </is>
+      </c>
+      <c r="C10" s="12">
+        <f>Rates!B11</f>
+        <v/>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>77.16</v>
+      </c>
+      <c r="E10" s="12">
+        <f>D10*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="12">
+        <f>C10-E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>C10/E10</f>
+        <v/>
+      </c>
+      <c r="H10" s="14">
+        <f>'Roster &amp; Hours'!L5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Taylor Nelson</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Engineer II</t>
+        </is>
+      </c>
+      <c r="C11" s="12">
+        <f>Rates!B12</f>
+        <v/>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>77.16</v>
+      </c>
+      <c r="E11" s="12">
+        <f>D11*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>C11-E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="21">
+        <f>C11/E11</f>
+        <v/>
+      </c>
+      <c r="H11" s="14">
+        <f>'Roster &amp; Hours'!L7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Collin Allen</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Graphics Technician</t>
+        </is>
+      </c>
+      <c r="C12" s="12">
+        <f>Rates!B6</f>
+        <v/>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>51.11</v>
+      </c>
+      <c r="E12" s="12">
+        <f>D12*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>C12-E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>C12/E12</f>
+        <v/>
+      </c>
+      <c r="H12" s="14">
+        <f>'Roster &amp; Hours'!L10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Randy Pynenberg</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Engineer IV</t>
+        </is>
+      </c>
+      <c r="C13" s="12">
+        <f>Rates!B14</f>
+        <v/>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="14">
+        <f>'Roster &amp; Hours'!L13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Auston Hopson</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Graphics Technician</t>
+        </is>
+      </c>
+      <c r="C14" s="12">
+        <f>Rates!B6</f>
+        <v/>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="14">
+        <f>'Roster &amp; Hours'!L14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Blended (weighted by billable hrs)</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="18">
+        <f>SUMPRODUCT('Roster &amp; Hours'!I5:I12,D5:D12)/SUM('Roster &amp; Hours'!I5:I12)</f>
+        <v/>
+      </c>
+      <c r="E15" s="18">
+        <f>D15*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="17" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>RAW vs BURDENED — assessment: these are base/pay rates, burden-EXCLUSIVE. Two tells:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. The GL books burden (FICA, UI, WC, health, pension, benefits, vac/hol = $157.4K YTD) as separate</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     operating-expense lines, NOT inside Cost of Revenues. If the job-cost rate were fully loaded, that</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     burden would sit in COGS instead — it cannot be in both. So the rate feeding COGS is burden-free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. On the COINS internal-labor job (9715), PTO, holiday and sick hours are booked at the SAME per-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     rate. A fully-burdened rate would double-count fringe when vacation/holiday time is also charged at it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Therefore: loaded cost = raw × (1 + burden%), burden ≈ 33.8% blended (Assumptions!B9). Note the blend is</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>approximate — health insurance is ~flat $/head (heavier on lower-paid staff) and payroll taxes cap on high</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>earners, so true burden % is higher at the bottom of the roster and lower at the top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TO CONFIRM DEFINITIVELY: ask payroll/COINS admin what the standard cost rate includes, or reconcile the</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>timesheet direct-labor total to the GL 'Labor-Design Services' line ($428.5K YTD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Cost rates cluster by grade (both Engineer IIIs = $107.60), a good validation. Taylor Nelson costs at the</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Engineer I rate ($77.16) despite the assumed Engineer II billing class — worth confirming.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3556,60 +4257,60 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="23" t="n">
         <v>110.5</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="23" t="n">
         <v>96.8</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="23" t="n">
         <v>39.3</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="23" t="n">
         <v>94.59999999999999</v>
       </c>
-      <c r="F5" s="21" t="n">
+      <c r="F5" s="23" t="n">
         <v>85.5</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="23" t="n">
         <v>124.4</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="24">
         <f>SUM(B5:G5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Cost of Sales (derived)</t>
         </is>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="23">
         <f>B5-B7</f>
         <v/>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="23">
         <f>C5-C7</f>
         <v/>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="23">
         <f>D5-D7</f>
         <v/>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="23">
         <f>E5-E7</f>
         <v/>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="23">
         <f>F5-F7</f>
         <v/>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="23">
         <f>G5-G7</f>
         <v/>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="24">
         <f>SUM(B6:G6)</f>
         <v/>
       </c>
@@ -3620,25 +4321,25 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="23" t="n">
         <v>52.6</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="23" t="n">
         <v>24.2</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="23" t="n">
         <v>-15.7</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="23" t="n">
         <v>33.7</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="23" t="n">
         <v>-18</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="23" t="n">
         <v>45.8</v>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="24">
         <f>SUM(B7:G7)</f>
         <v/>
       </c>
@@ -3649,66 +4350,66 @@
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="26">
         <f>B7/B5</f>
         <v/>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="26">
         <f>C7/C5</f>
         <v/>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="26">
         <f>D7/D5</f>
         <v/>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="26">
         <f>E7/E5</f>
         <v/>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="26">
         <f>F7/F5</f>
         <v/>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="26">
         <f>G7/G5</f>
         <v/>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="26">
         <f>H7/H5</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Operating Expenses (derived)</t>
         </is>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="23">
         <f>B7-B10</f>
         <v/>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="23">
         <f>C7-C10</f>
         <v/>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="23">
         <f>D7-D10</f>
         <v/>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="23">
         <f>E7-E10</f>
         <v/>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="23">
         <f>F7-F10</f>
         <v/>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="23">
         <f>G7-G10</f>
         <v/>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="24">
         <f>SUM(B9:G9)</f>
         <v/>
       </c>
@@ -3719,25 +4420,25 @@
           <t>Net Income / (Loss)</t>
         </is>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="23" t="n">
         <v>-41.7</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="23" t="n">
         <v>-49.1</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="23" t="n">
         <v>-98.8</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="23" t="n">
         <v>-60.5</v>
       </c>
-      <c r="F10" s="21" t="n">
+      <c r="F10" s="23" t="n">
         <v>-54.5</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="23" t="n">
         <v>-15.8</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="24">
         <f>SUM(B10:G10)</f>
         <v/>
       </c>
@@ -3748,31 +4449,31 @@
           <t>Net margin %</t>
         </is>
       </c>
-      <c r="B11" s="24">
+      <c r="B11" s="26">
         <f>B10/B5</f>
         <v/>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="26">
         <f>C10/C5</f>
         <v/>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="26">
         <f>D10/D5</f>
         <v/>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="26">
         <f>E10/E5</f>
         <v/>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="26">
         <f>F10/F5</f>
         <v/>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="26">
         <f>G10/G5</f>
         <v/>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="26">
         <f>H10/H5</f>
         <v/>
       </c>
@@ -3825,25 +4526,25 @@
           <t>Revenue — budget</t>
         </is>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14" s="23" t="n">
         <v>169.1</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="23" t="n">
         <v>169.1</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="23" t="n">
         <v>169.1</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="23" t="n">
         <v>169.1</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="23" t="n">
         <v>169.1</v>
       </c>
-      <c r="G14" s="21" t="n">
+      <c r="G14" s="23" t="n">
         <v>169.1</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="24">
         <f>SUM(B14:G14)</f>
         <v/>
       </c>
@@ -3854,25 +4555,25 @@
           <t>Gross Profit — budget</t>
         </is>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="23" t="n">
         <v>104.1</v>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="23" t="n">
         <v>104.1</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="23" t="n">
         <v>104.1</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="23" t="n">
         <v>104.2</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F15" s="23" t="n">
         <v>104.1</v>
       </c>
-      <c r="G15" s="21" t="n">
+      <c r="G15" s="23" t="n">
         <v>104.1</v>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="24">
         <f>SUM(B15:G15)</f>
         <v/>
       </c>
@@ -3883,25 +4584,25 @@
           <t>Net Income — budget</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="23" t="n">
         <v>11.6</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="23" t="n">
         <v>11.6</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="23" t="n">
         <v>11.7</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="23" t="n">
         <v>11.6</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="23" t="n">
         <v>11.6</v>
       </c>
-      <c r="G16" s="21" t="n">
+      <c r="G16" s="23" t="n">
         <v>11.6</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="24">
         <f>SUM(B16:G16)</f>
         <v/>
       </c>
@@ -3934,15 +4635,15 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="23">
         <f>H5</f>
         <v/>
       </c>
-      <c r="C19" s="21">
+      <c r="C19" s="23">
         <f>H14</f>
         <v/>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="23">
         <f>B19-C19</f>
         <v/>
       </c>
@@ -3953,15 +4654,15 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="23">
         <f>H7</f>
         <v/>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="23">
         <f>H15</f>
         <v/>
       </c>
-      <c r="D20" s="21">
+      <c r="D20" s="23">
         <f>B20-C20</f>
         <v/>
       </c>
@@ -3972,15 +4673,15 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="23">
         <f>H10</f>
         <v/>
       </c>
-      <c r="C21" s="21">
+      <c r="C21" s="23">
         <f>H16</f>
         <v/>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="23">
         <f>B21-C21</f>
         <v/>
       </c>
@@ -3997,7 +4698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4067,27 +4768,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Sales-Design Services</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="28" t="n">
         <v>124360</v>
       </c>
-      <c r="C5" s="26" t="n">
+      <c r="C5" s="28" t="n">
         <v>169094</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="D5" s="28" t="n">
         <v>86705</v>
       </c>
-      <c r="E5" s="26" t="n">
+      <c r="E5" s="28" t="n">
         <v>551013</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="28" t="n">
         <v>1014563</v>
       </c>
-      <c r="G5" s="26" t="n">
+      <c r="G5" s="28" t="n">
         <v>399143</v>
       </c>
     </row>
@@ -4142,52 +4843,52 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Direct Cost of Revenues Earned</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="28" t="n">
         <v>78573</v>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="28" t="n">
         <v>64980</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="D8" s="28" t="n">
         <v>43947</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E8" s="28" t="n">
         <v>428498</v>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="28" t="n">
         <v>389882</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="28" t="n">
         <v>680511</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="28" t="n">
         <v>45787</v>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="28" t="n">
         <v>104114</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="D9" s="28" t="n">
         <v>42757</v>
       </c>
-      <c r="E9" s="26" t="n">
+      <c r="E9" s="28" t="n">
         <v>122514</v>
       </c>
-      <c r="F9" s="26" t="n">
+      <c r="F9" s="28" t="n">
         <v>624681</v>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="28" t="n">
         <v>-281368</v>
       </c>
     </row>
@@ -5117,52 +5818,52 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25" t="inlineStr">
+      <c r="A47" s="27" t="inlineStr">
         <is>
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B47" s="26" t="n">
+      <c r="B47" s="28" t="n">
         <v>55620</v>
       </c>
-      <c r="C47" s="26" t="n">
+      <c r="C47" s="28" t="n">
         <v>92497</v>
       </c>
-      <c r="D47" s="26" t="n">
+      <c r="D47" s="28" t="n">
         <v>122857</v>
       </c>
-      <c r="E47" s="26" t="n">
+      <c r="E47" s="28" t="n">
         <v>412964</v>
       </c>
-      <c r="F47" s="26" t="n">
+      <c r="F47" s="28" t="n">
         <v>554982</v>
       </c>
-      <c r="G47" s="26" t="n">
+      <c r="G47" s="28" t="n">
         <v>612073</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="25" t="inlineStr">
+      <c r="A48" s="27" t="inlineStr">
         <is>
           <t>Operating Income (Loss)</t>
         </is>
       </c>
-      <c r="B48" s="26" t="n">
+      <c r="B48" s="28" t="n">
         <v>-9832</v>
       </c>
-      <c r="C48" s="26" t="n">
+      <c r="C48" s="28" t="n">
         <v>11617</v>
       </c>
-      <c r="D48" s="26" t="n">
+      <c r="D48" s="28" t="n">
         <v>-80100</v>
       </c>
-      <c r="E48" s="26" t="n">
+      <c r="E48" s="28" t="n">
         <v>-290450</v>
       </c>
-      <c r="F48" s="26" t="n">
+      <c r="F48" s="28" t="n">
         <v>69699</v>
       </c>
-      <c r="G48" s="26" t="n">
+      <c r="G48" s="28" t="n">
         <v>-893441</v>
       </c>
     </row>
@@ -5192,27 +5893,27 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="25" t="inlineStr">
+      <c r="A50" s="27" t="inlineStr">
         <is>
           <t>Net Income (Loss)</t>
         </is>
       </c>
-      <c r="B50" s="26" t="n">
+      <c r="B50" s="28" t="n">
         <v>-15845</v>
       </c>
-      <c r="C50" s="26" t="n">
+      <c r="C50" s="28" t="n">
         <v>11617</v>
       </c>
-      <c r="D50" s="26" t="n">
+      <c r="D50" s="28" t="n">
         <v>-84993</v>
       </c>
-      <c r="E50" s="26" t="n">
+      <c r="E50" s="28" t="n">
         <v>-320537</v>
       </c>
-      <c r="F50" s="26" t="n">
+      <c r="F50" s="28" t="n">
         <v>69699</v>
       </c>
-      <c r="G50" s="26" t="n">
+      <c r="G50" s="28" t="n">
         <v>-922542</v>
       </c>
     </row>
@@ -5222,27 +5923,27 @@
           <t>OILI (Operating Income less Interest)</t>
         </is>
       </c>
-      <c r="B51" s="27">
+      <c r="B51" s="29">
         <f>B48-B49</f>
         <v/>
       </c>
-      <c r="C51" s="27">
+      <c r="C51" s="29">
         <f>C48-C49</f>
         <v/>
       </c>
-      <c r="D51" s="27">
+      <c r="D51" s="29">
         <f>D48-D49</f>
         <v/>
       </c>
-      <c r="E51" s="27">
+      <c r="E51" s="29">
         <f>E48-E49</f>
         <v/>
       </c>
-      <c r="F51" s="27">
+      <c r="F51" s="29">
         <f>F48-F49</f>
         <v/>
       </c>
-      <c r="G51" s="27">
+      <c r="G51" s="29">
         <f>G48-G49</f>
         <v/>
       </c>
@@ -5253,27 +5954,27 @@
           <t>OILI return % (OILI ÷ revenue)</t>
         </is>
       </c>
-      <c r="B52" s="28">
+      <c r="B52" s="30">
         <f>IF(B5=0,"n/a",(B48-B49)/B5)</f>
         <v/>
       </c>
-      <c r="C52" s="28">
+      <c r="C52" s="30">
         <f>IF(C5=0,"n/a",(C48-C49)/C5)</f>
         <v/>
       </c>
-      <c r="D52" s="28">
+      <c r="D52" s="30">
         <f>IF(D5=0,"n/a",(D48-D49)/D5)</f>
         <v/>
       </c>
-      <c r="E52" s="28">
+      <c r="E52" s="30">
         <f>IF(E5=0,"n/a",(E48-E49)/E5)</f>
         <v/>
       </c>
-      <c r="F52" s="28">
+      <c r="F52" s="30">
         <f>IF(F5=0,"n/a",(F48-F49)/F5)</f>
         <v/>
       </c>
-      <c r="G52" s="28">
+      <c r="G52" s="30">
         <f>IF(G5=0,"n/a",(G48-G49)/G5)</f>
         <v/>
       </c>
@@ -5311,7 +6012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5407,13 +6108,13 @@
           <t>Total Current Assets</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="28" t="n">
         <v>141807</v>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="28" t="n">
         <v>46065</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="D8" s="28" t="n">
         <v>36000</v>
       </c>
     </row>
@@ -5439,13 +6140,13 @@
           <t>Total Assets</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="28" t="n">
         <v>141807</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="28" t="n">
         <v>46065</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="28" t="n">
         <v>36000</v>
       </c>
     </row>
@@ -5606,13 +6307,13 @@
           <t>Total Current Liabilities</t>
         </is>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="28" t="n">
         <v>52544</v>
       </c>
-      <c r="C21" s="26" t="n">
+      <c r="C21" s="28" t="n">
         <v>106898</v>
       </c>
-      <c r="D21" s="26" t="n">
+      <c r="D21" s="28" t="n">
         <v>121740</v>
       </c>
     </row>
@@ -5638,13 +6339,13 @@
           <t>Total Liabilities</t>
         </is>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="28" t="n">
         <v>3489166</v>
       </c>
-      <c r="C23" s="26" t="n">
+      <c r="C23" s="28" t="n">
         <v>3508376</v>
       </c>
-      <c r="D23" s="26" t="n">
+      <c r="D23" s="28" t="n">
         <v>2923425</v>
       </c>
     </row>
@@ -5709,13 +6410,13 @@
           <t>Total Shareholders' Equity</t>
         </is>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="28" t="n">
         <v>-3347360</v>
       </c>
-      <c r="C28" s="26" t="n">
+      <c r="C28" s="28" t="n">
         <v>-3462311</v>
       </c>
-      <c r="D28" s="26" t="n">
+      <c r="D28" s="28" t="n">
         <v>-2887425</v>
       </c>
     </row>
@@ -5725,13 +6426,13 @@
           <t>Total Liabilities &amp; Equity</t>
         </is>
       </c>
-      <c r="B29" s="26" t="n">
+      <c r="B29" s="28" t="n">
         <v>141807</v>
       </c>
-      <c r="C29" s="26" t="n">
+      <c r="C29" s="28" t="n">
         <v>46065</v>
       </c>
-      <c r="D29" s="26" t="n">
+      <c r="D29" s="28" t="n">
         <v>36000</v>
       </c>
     </row>
@@ -5768,7 +6469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5872,10 +6573,10 @@
           <t>Net Cash from Operating Activities</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="28" t="n">
         <v>-477155</v>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="28" t="n">
         <v>157782</v>
       </c>
     </row>
@@ -5898,10 +6599,10 @@
           <t>Net Change in Cash</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6080,7 +6781,7 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B24" s="26">
+      <c r="B24" s="28">
         <f>SUM(B17:B23)</f>
         <v/>
       </c>
@@ -6091,7 +6792,7 @@
           <t>Intercompany (HWC) share</t>
         </is>
       </c>
-      <c r="B25" s="24">
+      <c r="B25" s="26">
         <f>(B18+B19)/B24</f>
         <v/>
       </c>
@@ -6102,7 +6803,7 @@
           <t>CenterPoint share</t>
         </is>
       </c>
-      <c r="B26" s="24">
+      <c r="B26" s="26">
         <f>B17/B24</f>
         <v/>
       </c>
@@ -6111,164 +6812,6 @@
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Answers a Phase-1 question: CVR hours on HWC jobs ARE revenue-credited as intercompany sales (~20% of YTD revenue). CenterPoint is ~70% of revenue — matching its ~70% share of billable hours.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>HWC EPC — Baseline, January–May 2026 (all figures $K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Context for the engineering P&amp;L: design quality and constructability directly affect these outcomes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>HWC EPC ($K)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Apr</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>YTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>732.2</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>207.7</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>-321</v>
-      </c>
-      <c r="E5" s="21" t="n">
-        <v>-125.1</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>678.6</v>
-      </c>
-      <c r="G5" s="22">
-        <f>SUM(B5:F5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Net Profit / (Loss)</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>-318.3</v>
-      </c>
-      <c r="C6" s="21" t="n">
-        <v>-346.9</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <v>-672.8</v>
-      </c>
-      <c r="E6" s="21" t="n">
-        <v>-656.5</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <v>-114.8</v>
-      </c>
-      <c r="G6" s="22">
-        <f>SUM(B6:F6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Net margin % (YTD)</t>
-        </is>
-      </c>
-      <c r="G7" s="24">
-        <f>G6/G5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Negative revenue in March and April are billing adjustments/write-downs per the KPI report charts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Active EPC scorecard jobs (7/11/2026): 4 substation projects, PO $4.3M–$6.6M, plan margins 12.7%–16.4%,</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>cost variance +3.6% to −19.8%. Engineering share of paired EPC pursuits runs ~4–5% of EPC job value.</t>
         </is>
       </c>
     </row>

</xml_diff>